<commit_message>
Update RGU faculty rooms data and dashboard calculations to match updated RGU.xlsx
</commit_message>
<xml_diff>
--- a/RGU.xlsx
+++ b/RGU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\CLASS ROOM\2027-28\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Class Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{932329CC-8673-4566-B23F-3942C9FD8CE2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5606C85E-D8D9-4407-9EEC-4222122A089E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,21 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="51">
   <si>
     <t>Academic Year 2027-2028</t>
   </si>
@@ -173,11 +182,16 @@
 3. No.of Classrooms School of Law : 3</t>
   </si>
   <si>
-    <t>Note :
-1. No.of faculty rooms required for 2026-2027 : 0
-2. Moot Court : 1
-3. No.of Staff Room School of Law : 1
-4. School of Law Couselling Room : 1</t>
+    <t>No.of Staff Room School of Law : 1</t>
+  </si>
+  <si>
+    <t>School of Law Couselling Room : 1</t>
+  </si>
+  <si>
+    <t>Required for 2026-2027 is below</t>
+  </si>
+  <si>
+    <t>Moot Court : 1</t>
   </si>
 </sst>
 </file>
@@ -245,7 +259,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -264,11 +278,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -293,9 +306,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -587,232 +597,232 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F46"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F49"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
-    <col min="2" max="2" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.140625" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" customWidth="1"/>
-    <col min="6" max="6" width="23.5703125" customWidth="1"/>
+    <col min="2" max="2" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.109375" customWidth="1"/>
+    <col min="5" max="5" width="11.33203125" customWidth="1"/>
+    <col min="6" max="6" width="23.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B2" s="20" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B2" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="20" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C2" s="18" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="20">
+      <c r="B3" s="18">
         <v>2243</v>
       </c>
-      <c r="C3" s="20">
+      <c r="C3" s="18">
         <v>2680</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="20">
+      <c r="B4" s="18">
         <v>5200</v>
       </c>
-      <c r="C4" s="20">
+      <c r="C4" s="18">
         <v>5260</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="20">
+      <c r="B6" s="18">
         <v>3300</v>
       </c>
-      <c r="C6" s="20">
+      <c r="C6" s="18">
         <v>3300</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="20">
+      <c r="B7" s="18">
         <f>2498-200</f>
         <v>2298</v>
       </c>
-      <c r="C7" s="20">
+      <c r="C7" s="18">
         <v>3300</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="20">
+      <c r="B8" s="18">
         <f>1910-100</f>
         <v>1810</v>
       </c>
-      <c r="C8" s="20">
+      <c r="C8" s="18">
         <v>2298</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="20">
+      <c r="B9" s="18">
         <v>270</v>
       </c>
-      <c r="C9" s="20">
+      <c r="C9" s="18">
         <v>300</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="20">
+      <c r="B10" s="18">
         <v>500</v>
       </c>
-      <c r="C10" s="20">
+      <c r="C10" s="18">
         <v>500</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B11" s="20">
+      <c r="B11" s="18">
         <v>400</v>
       </c>
-      <c r="C11" s="20">
+      <c r="C11" s="18">
         <v>500</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="20">
+      <c r="B12" s="18">
         <v>720</v>
       </c>
-      <c r="C12" s="20">
+      <c r="C12" s="18">
         <v>1080</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="20">
+      <c r="B13" s="18">
         <v>600</v>
       </c>
-      <c r="C13" s="20">
+      <c r="C13" s="18">
         <v>1020</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="20">
+      <c r="B14" s="18">
         <v>500</v>
       </c>
-      <c r="C14" s="20">
+      <c r="C14" s="18">
         <v>800</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="20">
+      <c r="B15" s="18">
         <v>500</v>
       </c>
-      <c r="C15" s="20">
+      <c r="C15" s="18">
         <v>600</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="20">
+      <c r="B16" s="18">
         <v>120</v>
       </c>
-      <c r="C16" s="20">
+      <c r="C16" s="18">
         <v>120</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="20">
+      <c r="B17" s="18">
         <v>60</v>
       </c>
-      <c r="C17" s="20">
+      <c r="C17" s="18">
         <v>60</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="21">
+      <c r="B18" s="19">
         <f>SUM(B6:B17)</f>
         <v>11078</v>
       </c>
-      <c r="C18" s="21">
+      <c r="C18" s="19">
         <f>SUM(C6:C17)</f>
         <v>13878</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:6" s="19" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
+    <row r="21" spans="1:6" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D21" s="17" t="s">
+      <c r="D21" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="E21" s="18" t="s">
+      <c r="E21" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="F21" s="18" t="s">
+      <c r="F21" s="17" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
         <v>12</v>
       </c>
@@ -834,7 +844,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
         <v>13</v>
       </c>
@@ -855,7 +865,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
         <v>14</v>
       </c>
@@ -876,7 +886,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
         <v>20</v>
       </c>
@@ -898,7 +908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
         <v>21</v>
       </c>
@@ -920,7 +930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
         <v>22</v>
       </c>
@@ -942,42 +952,42 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" s="8" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
+    <row r="28" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B28" s="9"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="s">
         <v>25</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C31" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D31" s="13" t="s">
+      <c r="D31" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="E31" s="22" t="s">
+      <c r="E31" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="F31" s="22" t="s">
+      <c r="F31" s="20" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
         <v>43</v>
       </c>
@@ -999,7 +1009,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
         <v>44</v>
       </c>
@@ -1021,7 +1031,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
         <v>26</v>
       </c>
@@ -1043,35 +1053,35 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A35" s="10" t="s">
+    <row r="35" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A35" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="38" spans="1:6" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A38" s="11"/>
-      <c r="B38" s="12" t="s">
+    <row r="38" spans="1:6" s="13" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="10"/>
+      <c r="B38" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C38" s="13" t="s">
+      <c r="C38" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D38" s="13" t="s">
+      <c r="D38" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="E38" s="22" t="s">
+      <c r="E38" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="F38" s="22" t="s">
+      <c r="F38" s="20" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="7" t="s">
         <v>30</v>
       </c>
@@ -1093,7 +1103,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
         <v>31</v>
       </c>
@@ -1115,71 +1125,91 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="90" x14ac:dyDescent="0.25">
-      <c r="A41" s="10" t="s">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B41" s="3"/>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="6"/>
+      <c r="F41" s="6"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" s="10" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="s">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="44" spans="1:6" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A44" s="11"/>
-      <c r="B44" s="12" t="s">
+    <row r="47" spans="1:6" s="13" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A47" s="10"/>
+      <c r="B47" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C44" s="13" t="s">
+      <c r="C47" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D44" s="13" t="s">
+      <c r="D47" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="E44" s="22" t="s">
+      <c r="E47" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="F44" s="22" t="s">
+      <c r="F47" s="20" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="7" t="s">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B45" s="3">
+      <c r="B48" s="3">
         <v>0</v>
       </c>
-      <c r="C45" s="5">
-        <v>1</v>
-      </c>
-      <c r="D45" s="5">
-        <v>1</v>
-      </c>
-      <c r="E45" s="6">
-        <v>1</v>
-      </c>
-      <c r="F45" s="6">
+      <c r="C48" s="5">
+        <v>1</v>
+      </c>
+      <c r="D48" s="5">
+        <v>1</v>
+      </c>
+      <c r="E48" s="6">
+        <v>1</v>
+      </c>
+      <c r="F48" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="7" t="s">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B46" s="3">
+      <c r="B49" s="3">
         <v>0</v>
       </c>
-      <c r="C46" s="5">
-        <v>1</v>
-      </c>
-      <c r="D46" s="5">
-        <v>1</v>
-      </c>
-      <c r="E46" s="6">
-        <v>1</v>
-      </c>
-      <c r="F46" s="6">
+      <c r="C49" s="5">
+        <v>1</v>
+      </c>
+      <c r="D49" s="5">
+        <v>1</v>
+      </c>
+      <c r="E49" s="6">
+        <v>1</v>
+      </c>
+      <c r="F49" s="6">
         <v>0</v>
       </c>
     </row>

</xml_diff>